<commit_message>
chore: update pyspark problem list in spreadsheet
</commit_message>
<xml_diff>
--- a/problems/pyspark_120_problems.xlsx
+++ b/problems/pyspark_120_problems.xlsx
@@ -5556,7 +5556,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -5578,7 +5578,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -5600,7 +5600,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -5622,7 +5622,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -5644,7 +5644,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -5666,7 +5666,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{"departments": "departments"}</t>
+          <t>departments:departments</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -5688,7 +5688,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -5710,7 +5710,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -5732,7 +5732,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -5754,7 +5754,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -5798,7 +5798,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>{"departments": "departments"}</t>
+          <t>departments:departments</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -5820,7 +5820,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>{"sales": "sales"}</t>
+          <t>sales:sales</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -5886,7 +5886,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>{"products": "products"}</t>
+          <t>products:products</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>{"products": "products"}</t>
+          <t>products:products</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -5930,7 +5930,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>{"web_logs": "web_logs"}</t>
+          <t>web_logs:web_logs</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>{"sales": "sales"}</t>
+          <t>sales:sales</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -5996,7 +5996,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -6018,7 +6018,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -6040,7 +6040,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>{"sales": "sales"}</t>
+          <t>sales:sales</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -6062,7 +6062,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>{"sales": "sales"}</t>
+          <t>sales:sales</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -6084,7 +6084,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>{"products": "products"}</t>
+          <t>products:products</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -6106,7 +6106,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -6128,7 +6128,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>{"sales": "sales"}</t>
+          <t>sales:sales</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -6172,7 +6172,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>{"sales": "sales"}</t>
+          <t>sales:sales</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -6194,7 +6194,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>{"web_logs": "web_logs"}</t>
+          <t>web_logs:web_logs</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -6216,7 +6216,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -6238,7 +6238,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>{"sales": "sales"}</t>
+          <t>sales:sales</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -6260,7 +6260,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -6304,7 +6304,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>{"products": "products"}</t>
+          <t>products:products</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -6326,7 +6326,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -6348,7 +6348,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>{"sales": "sales"}</t>
+          <t>sales:sales</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -6370,7 +6370,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>{"web_logs": "web_logs"}</t>
+          <t>web_logs:web_logs</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -6392,7 +6392,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>{"sales": "sales"}</t>
+          <t>sales:sales</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -6436,7 +6436,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>{"employees": "employees", "departments": "departments"}</t>
+          <t>employees:employees,departments:departments</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>{"employees": "employees", "departments": "departments"}</t>
+          <t>employees:employees,departments:departments</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>{"sales": "sales", "products": "products"}</t>
+          <t>sales:sales,products:products</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -6502,7 +6502,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>{"employees": "employees", "departments": "departments"}</t>
+          <t>employees:employees,departments:departments</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -6524,7 +6524,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>{"employees": "employees", "departments": "departments"}</t>
+          <t>employees:employees,departments:departments</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -6546,7 +6546,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>{"sales": "sales", "products": "products"}</t>
+          <t>sales:sales,products:products</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -6568,7 +6568,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>{"employees": "employees", "departments": "departments"}</t>
+          <t>employees:employees,departments:departments</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -6590,7 +6590,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>{"sales": "sales", "products": "products"}</t>
+          <t>sales:sales,products:products</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -6612,7 +6612,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -6634,7 +6634,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>{"employees": "employees", "departments": "departments"}</t>
+          <t>employees:employees,departments:departments</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -6678,7 +6678,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>{"employees": "employees", "departments": "departments"}</t>
+          <t>employees:employees,departments:departments</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -6700,7 +6700,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>{"products": "products", "sales": "sales"}</t>
+          <t>products:products,sales:sales</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -6722,7 +6722,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>{"employees": "employees", "departments": "departments"}</t>
+          <t>employees:employees,departments:departments</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -6744,7 +6744,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>{"employees": "employees", "departments": "departments"}</t>
+          <t>employees:employees,departments:departments</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -6766,7 +6766,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>{"employees": "employees", "departments": "departments"}</t>
+          <t>employees:employees,departments:departments</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -6788,7 +6788,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>{"products": "products", "sales": "sales"}</t>
+          <t>products:products,sales:sales</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -6810,7 +6810,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>{"products": "products", "sales": "sales"}</t>
+          <t>products:products,sales:sales</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -6832,7 +6832,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>{"employees": "employees", "departments": "departments"}</t>
+          <t>employees:employees,departments:departments</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -6854,7 +6854,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>{"employees": "employees", "departments": "departments"}</t>
+          <t>employees:employees,departments:departments</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -6876,7 +6876,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -6898,7 +6898,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>{"sales": "sales"}</t>
+          <t>sales:sales</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -6942,7 +6942,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>{"sales": "sales"}</t>
+          <t>sales:sales</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -6986,7 +6986,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>{"sales": "sales"}</t>
+          <t>sales:sales</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -7030,7 +7030,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -7052,7 +7052,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -7074,7 +7074,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -7096,7 +7096,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -7118,7 +7118,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -7162,7 +7162,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -7206,7 +7206,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -7228,7 +7228,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -7250,7 +7250,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -7272,7 +7272,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -7294,7 +7294,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -7316,7 +7316,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -7338,7 +7338,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -7382,7 +7382,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -7404,7 +7404,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -7426,7 +7426,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -7448,7 +7448,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -7470,7 +7470,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -7492,7 +7492,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>{"products": "products"}</t>
+          <t>products:products</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -7536,7 +7536,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -7580,7 +7580,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -7602,7 +7602,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -7624,7 +7624,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -7646,7 +7646,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -7668,7 +7668,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -7690,7 +7690,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -7712,7 +7712,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -7734,7 +7734,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -7756,7 +7756,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -7778,7 +7778,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>{"sales": "sales"}</t>
+          <t>sales:sales</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -7800,7 +7800,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>{"employees": "employees", "departments": "departments"}</t>
+          <t>employees:employees,departments:departments</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -7822,7 +7822,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>{"departments": "departments"}</t>
+          <t>departments:departments</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -7866,7 +7866,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -7888,7 +7888,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -7910,7 +7910,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -7932,7 +7932,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -7954,7 +7954,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -7998,7 +7998,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -8020,7 +8020,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -8042,7 +8042,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -8086,7 +8086,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -8108,7 +8108,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -8130,7 +8130,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -8152,7 +8152,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -8174,7 +8174,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>{"employees": "employees"}</t>
+          <t>employees:employees</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">

</xml_diff>